<commit_message>
Revise HCM notebook to follow paper-style regression
</commit_message>
<xml_diff>
--- a/Data_folder/Hyperspherical_Confidence_Mapping(HCM)/Matrix Evaluation.xlsx
+++ b/Data_folder/Hyperspherical_Confidence_Mapping(HCM)/Matrix Evaluation.xlsx
@@ -14,33 +14,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Model</t>
   </si>
   <si>
+    <t>Cov@1Sigma</t>
+  </si>
+  <si>
+    <t>Cov@2Sigma</t>
+  </si>
+  <si>
+    <t>Cov@3Sigma</t>
+  </si>
+  <si>
+    <t>Pearson</t>
+  </si>
+  <si>
+    <t>Spearman</t>
+  </si>
+  <si>
+    <t>ECE_reg</t>
+  </si>
+  <si>
     <t>RMSE</t>
   </si>
   <si>
     <t>MAE</t>
   </si>
   <si>
-    <t>Pearson</t>
-  </si>
-  <si>
-    <t>Spearman</t>
-  </si>
-  <si>
-    <t>Coverage_95</t>
-  </si>
-  <si>
-    <t>Average_Interval_Width</t>
-  </si>
-  <si>
-    <t>Sharpness</t>
-  </si>
-  <si>
-    <t>Mean_Norm_Violation</t>
+    <t>Mean_Sigma_Hat</t>
+  </si>
+  <si>
+    <t>Mean_RawUncertainty</t>
   </si>
   <si>
     <t>HCM</t>
@@ -401,10 +407,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -432,34 +438,46 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2">
-        <v>11.35642746748372</v>
+        <v>0.6125</v>
       </c>
       <c r="C2">
-        <v>10.38754653930664</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>-0.09257794760375861</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>-0.00642287857477731</v>
+        <v>0.6463973074329308</v>
       </c>
       <c r="F2">
-        <v>0.9375</v>
+        <v>0.6742381622128458</v>
       </c>
       <c r="G2">
-        <v>171.4127502441406</v>
+        <v>1.677634118217975</v>
       </c>
       <c r="H2">
-        <v>43.72773742675781</v>
+        <v>12.40494251808339</v>
       </c>
       <c r="I2">
-        <v>0.1415259540081024</v>
+        <v>11.4947681427002</v>
+      </c>
+      <c r="J2">
+        <v>12.62805843353271</v>
+      </c>
+      <c r="K2">
+        <v>0.09807904809713364</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine HCM outputs for original scale and 95 interval
</commit_message>
<xml_diff>
--- a/Data_folder/Hyperspherical_Confidence_Mapping(HCM)/Matrix Evaluation.xlsx
+++ b/Data_folder/Hyperspherical_Confidence_Mapping(HCM)/Matrix Evaluation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Model</t>
   </si>
@@ -26,6 +26,12 @@
   </si>
   <si>
     <t>Cov@3Sigma</t>
+  </si>
+  <si>
+    <t>Coverage_95Interval</t>
+  </si>
+  <si>
+    <t>Average_95Interval_Width</t>
   </si>
   <si>
     <t>Pearson</t>
@@ -56,16 +62,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -81,7 +79,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -89,30 +87,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -407,77 +387,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B2">
-        <v>0.6125</v>
+        <v>0.575</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0.875</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>0.975</v>
       </c>
       <c r="E2">
-        <v>0.6463973074329308</v>
+        <v>0.875</v>
       </c>
       <c r="F2">
-        <v>0.6742381622128458</v>
+        <v>14.82101588438003</v>
       </c>
       <c r="G2">
-        <v>1.677634118217975</v>
+        <v>0.1597591534738199</v>
       </c>
       <c r="H2">
-        <v>12.40494251808339</v>
+        <v>0.2029535864978903</v>
       </c>
       <c r="I2">
-        <v>11.4947681427002</v>
+        <v>1.19296941489228</v>
       </c>
       <c r="J2">
-        <v>12.62805843353271</v>
+        <v>4.710181302340576</v>
       </c>
       <c r="K2">
-        <v>0.09807904809713364</v>
+        <v>3.811976477708738</v>
+      </c>
+      <c r="L2">
+        <v>3.780871399076538</v>
+      </c>
+      <c r="M2">
+        <v>0.4571174115085759</v>
       </c>
     </row>
   </sheetData>

</xml_diff>